<commit_message>
Friday GIS session: add Geomatica as presenter
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CAFC 2026 Agenda - All Sessions.xlsx
+++ b/docs/CAFC 2026 Agenda - All Sessions.xlsx
@@ -3128,7 +3128,11 @@
           <t>The Impact of GIS in the Caribbean</t>
         </is>
       </c>
-      <c r="C150" s="2" t="inlineStr"/>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Geomatica</t>
+        </is>
+      </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
           <t>Business Track</t>

</xml_diff>